<commit_message>
Read per-container plant arrival dates from ATP
Recognize ATP as the preferred import header, retain legacy aliases, and update synthetic fixtures and IT documentation. Reader tests pass with the ATP workbook.
</commit_message>
<xml_diff>
--- a/samples/importaciones_ficticias.xlsx
+++ b/samples/importaciones_ficticias.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +48,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -493,7 +493,7 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Llegada a planta</t>
+          <t>ATP</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,6 @@
           <t>In transit</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>HBL-EJEMPLO-001</t>
@@ -519,22 +518,16 @@
           <t>TTIU1000000</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>46294</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="I2" s="2" t="n">
         <v>46302</v>
       </c>
       <c r="J2" t="n">
         <v>40</v>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" s="1" t="n">
+      <c r="O2" s="2" t="n">
         <v>46300</v>
       </c>
     </row>
@@ -549,7 +542,6 @@
           <t>In transit</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>HBL-EJEMPLO-002</t>
@@ -560,22 +552,16 @@
           <t>TTIU1000001</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>46294</v>
       </c>
-      <c r="I3" s="1" t="n">
+      <c r="I3" s="2" t="n">
         <v>46302</v>
       </c>
       <c r="J3" t="n">
         <v>40</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" s="1" t="n">
+      <c r="O3" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -585,24 +571,15 @@
           <t>Partes de motores</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>TTIU1000002</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" s="1" t="n"/>
-      <c r="I4" s="1" t="n"/>
       <c r="J4" t="n">
         <v>40</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" s="1" t="n">
+      <c r="O4" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -612,24 +589,15 @@
           <t>Plywood</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>TTIU1000003</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" s="1" t="n"/>
-      <c r="I5" s="1" t="n"/>
       <c r="J5" t="n">
         <v>40</v>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" s="1" t="n">
+      <c r="O5" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -639,24 +607,15 @@
           <t>Partes de motores</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>TTIU1000004</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" s="1" t="n"/>
-      <c r="I6" s="1" t="n"/>
       <c r="J6" t="n">
         <v>40</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" s="1" t="n">
+      <c r="O6" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -666,24 +625,15 @@
           <t>Partes de motores</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>TTIU1000005</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" s="1" t="n"/>
-      <c r="I7" s="1" t="n"/>
       <c r="J7" t="n">
         <v>40</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" s="1" t="n">
+      <c r="O7" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -693,24 +643,15 @@
           <t>Plywood</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>TTIU1000006</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" s="1" t="n"/>
-      <c r="I8" s="1" t="n"/>
       <c r="J8" t="n">
         <v>40</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" s="1" t="n">
+      <c r="O8" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -725,7 +666,6 @@
           <t>In transit</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>HBL-EJEMPLO-003</t>
@@ -736,22 +676,16 @@
           <t>TTIU1000007</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>46294</v>
       </c>
-      <c r="I9" s="1" t="n">
+      <c r="I9" s="2" t="n">
         <v>46302</v>
       </c>
       <c r="J9" t="n">
         <v>40</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" s="1" t="n">
+      <c r="O9" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -761,24 +695,15 @@
           <t>Partes de motores</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>TTIU1000008</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" s="1" t="n"/>
-      <c r="I10" s="1" t="n"/>
       <c r="J10" t="n">
         <v>40</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" s="1" t="n">
+      <c r="O10" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -788,24 +713,15 @@
           <t>Plywood</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>TTIU1000009</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" s="1" t="n"/>
-      <c r="I11" s="1" t="n"/>
       <c r="J11" t="n">
         <v>40</v>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" s="1" t="n">
+      <c r="O11" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -815,24 +731,15 @@
           <t>Partes de motores</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>TTIU1000010</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" s="1" t="n"/>
-      <c r="I12" s="1" t="n"/>
       <c r="J12" t="n">
         <v>40</v>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" s="1" t="n">
+      <c r="O12" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -842,24 +749,15 @@
           <t>Partes de motores</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>TTIU1000011</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" s="1" t="n"/>
-      <c r="I13" s="1" t="n"/>
       <c r="J13" t="n">
         <v>40</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" s="1" t="n">
+      <c r="O13" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -869,24 +767,15 @@
           <t>Plywood</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>TTIU1000012</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" s="1" t="n"/>
-      <c r="I14" s="1" t="n"/>
       <c r="J14" t="n">
         <v>40</v>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" s="1" t="n">
+      <c r="O14" s="2" t="n">
         <v>46301</v>
       </c>
     </row>
@@ -911,11 +800,11 @@
           <t>TTIU1999999</t>
         </is>
       </c>
-      <c r="H15" s="1" t="n"/>
-      <c r="I15" s="1" t="n">
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n">
         <v>46297</v>
       </c>
-      <c r="O15" s="1" t="n">
+      <c r="O15" s="2" t="n">
         <v>46300</v>
       </c>
     </row>
@@ -940,11 +829,11 @@
           <t>TTIU1888888</t>
         </is>
       </c>
-      <c r="H16" s="1" t="n"/>
-      <c r="I16" s="1" t="n">
-        <v>46301</v>
-      </c>
-      <c r="O16" s="1" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="O16" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>